<commit_message>
Update enterprise Excel reports, HTML dashboards, test summaries, and screenshots for 500+ test cases
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Passed_Test_Cases.xlsx
+++ b/Test Results/Excel/Passed_Test_Cases.xlsx
@@ -430,7 +430,7 @@
         <v>LOW</v>
       </c>
       <c r="E2" t="str">
-        <v>0.059s</v>
+        <v>0.137s</v>
       </c>
     </row>
     <row r="3">
@@ -447,7 +447,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E3" t="str">
-        <v>0.153s</v>
+        <v>0.143s</v>
       </c>
     </row>
     <row r="4">
@@ -464,7 +464,7 @@
         <v>HIGH</v>
       </c>
       <c r="E4" t="str">
-        <v>0.108s</v>
+        <v>0.117s</v>
       </c>
     </row>
     <row r="5">
@@ -481,7 +481,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E5" t="str">
-        <v>0.140s</v>
+        <v>0.057s</v>
       </c>
     </row>
     <row r="6">
@@ -498,7 +498,7 @@
         <v>LOW</v>
       </c>
       <c r="E6" t="str">
-        <v>0.096s</v>
+        <v>0.118s</v>
       </c>
     </row>
     <row r="7">
@@ -515,7 +515,7 @@
         <v>HIGH</v>
       </c>
       <c r="E7" t="str">
-        <v>0.069s</v>
+        <v>0.064s</v>
       </c>
     </row>
     <row r="8">
@@ -532,7 +532,7 @@
         <v>LOW</v>
       </c>
       <c r="E8" t="str">
-        <v>0.068s</v>
+        <v>0.070s</v>
       </c>
     </row>
     <row r="9">
@@ -549,7 +549,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E9" t="str">
-        <v>0.057s</v>
+        <v>0.069s</v>
       </c>
     </row>
     <row r="10">
@@ -566,7 +566,7 @@
         <v>HIGH</v>
       </c>
       <c r="E10" t="str">
-        <v>0.094s</v>
+        <v>0.137s</v>
       </c>
     </row>
     <row r="11">
@@ -583,7 +583,7 @@
         <v>LOW</v>
       </c>
       <c r="E11" t="str">
-        <v>0.143s</v>
+        <v>0.093s</v>
       </c>
     </row>
     <row r="12">
@@ -600,7 +600,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E12" t="str">
-        <v>0.056s</v>
+        <v>0.044s</v>
       </c>
     </row>
     <row r="13">
@@ -617,7 +617,7 @@
         <v>LOW</v>
       </c>
       <c r="E13" t="str">
-        <v>0.155s</v>
+        <v>0.059s</v>
       </c>
     </row>
     <row r="14">
@@ -634,7 +634,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E14" t="str">
-        <v>0.043s</v>
+        <v>0.065s</v>
       </c>
     </row>
     <row r="15">
@@ -651,7 +651,7 @@
         <v>HIGH</v>
       </c>
       <c r="E15" t="str">
-        <v>0.060s</v>
+        <v>0.097s</v>
       </c>
     </row>
     <row r="16">
@@ -668,7 +668,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E16" t="str">
-        <v>0.113s</v>
+        <v>0.076s</v>
       </c>
     </row>
     <row r="17">
@@ -685,7 +685,7 @@
         <v>LOW</v>
       </c>
       <c r="E17" t="str">
-        <v>0.060s</v>
+        <v>0.087s</v>
       </c>
     </row>
     <row r="18">
@@ -702,7 +702,7 @@
         <v>HIGH</v>
       </c>
       <c r="E18" t="str">
-        <v>0.057s</v>
+        <v>0.146s</v>
       </c>
     </row>
     <row r="19">
@@ -719,7 +719,7 @@
         <v>LOW</v>
       </c>
       <c r="E19" t="str">
-        <v>0.141s</v>
+        <v>0.100s</v>
       </c>
     </row>
     <row r="20">
@@ -736,7 +736,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E20" t="str">
-        <v>0.119s</v>
+        <v>0.043s</v>
       </c>
     </row>
     <row r="21">
@@ -753,7 +753,7 @@
         <v>HIGH</v>
       </c>
       <c r="E21" t="str">
-        <v>0.109s</v>
+        <v>0.148s</v>
       </c>
     </row>
     <row r="22">
@@ -770,7 +770,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E22" t="str">
-        <v>0.073s</v>
+        <v>0.095s</v>
       </c>
     </row>
     <row r="23">
@@ -787,7 +787,7 @@
         <v>LOW</v>
       </c>
       <c r="E23" t="str">
-        <v>0.083s</v>
+        <v>0.082s</v>
       </c>
     </row>
     <row r="24">
@@ -804,7 +804,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E24" t="str">
-        <v>0.047s</v>
+        <v>0.055s</v>
       </c>
     </row>
     <row r="25">
@@ -821,7 +821,7 @@
         <v>LOW</v>
       </c>
       <c r="E25" t="str">
-        <v>0.047s</v>
+        <v>0.149s</v>
       </c>
     </row>
     <row r="26">
@@ -838,7 +838,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E26" t="str">
-        <v>0.095s</v>
+        <v>0.044s</v>
       </c>
     </row>
     <row r="27">
@@ -872,7 +872,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E28" t="str">
-        <v>0.044s</v>
+        <v>0.073s</v>
       </c>
     </row>
     <row r="29">
@@ -889,7 +889,7 @@
         <v>LOW</v>
       </c>
       <c r="E29" t="str">
-        <v>0.160s</v>
+        <v>0.106s</v>
       </c>
     </row>
     <row r="30">
@@ -906,7 +906,7 @@
         <v>HIGH</v>
       </c>
       <c r="E30" t="str">
-        <v>0.090s</v>
+        <v>0.066s</v>
       </c>
     </row>
     <row r="31">
@@ -923,7 +923,7 @@
         <v>LOW</v>
       </c>
       <c r="E31" t="str">
-        <v>0.051s</v>
+        <v>0.151s</v>
       </c>
     </row>
     <row r="32">
@@ -940,7 +940,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E32" t="str">
-        <v>0.063s</v>
+        <v>0.088s</v>
       </c>
     </row>
     <row r="33">
@@ -957,7 +957,7 @@
         <v>HIGH</v>
       </c>
       <c r="E33" t="str">
-        <v>0.081s</v>
+        <v>0.125s</v>
       </c>
     </row>
     <row r="34">
@@ -974,7 +974,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E34" t="str">
-        <v>0.141s</v>
+        <v>0.067s</v>
       </c>
     </row>
     <row r="35">
@@ -991,7 +991,7 @@
         <v>LOW</v>
       </c>
       <c r="E35" t="str">
-        <v>0.077s</v>
+        <v>0.102s</v>
       </c>
     </row>
     <row r="36">
@@ -1008,7 +1008,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E36" t="str">
-        <v>0.066s</v>
+        <v>0.153s</v>
       </c>
     </row>
     <row r="37">
@@ -1025,7 +1025,7 @@
         <v>LOW</v>
       </c>
       <c r="E37" t="str">
-        <v>0.133s</v>
+        <v>0.071s</v>
       </c>
     </row>
     <row r="38">
@@ -1042,7 +1042,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E38" t="str">
-        <v>0.153s</v>
+        <v>0.134s</v>
       </c>
     </row>
     <row r="39">
@@ -1059,7 +1059,7 @@
         <v>HIGH</v>
       </c>
       <c r="E39" t="str">
-        <v>0.061s</v>
+        <v>0.084s</v>
       </c>
     </row>
     <row r="40">
@@ -1076,7 +1076,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E40" t="str">
-        <v>0.120s</v>
+        <v>0.099s</v>
       </c>
     </row>
     <row r="41">
@@ -1093,7 +1093,7 @@
         <v>LOW</v>
       </c>
       <c r="E41" t="str">
-        <v>0.095s</v>
+        <v>0.055s</v>
       </c>
     </row>
     <row r="42">
@@ -1110,7 +1110,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E42" t="str">
-        <v>0.077s</v>
+        <v>0.075s</v>
       </c>
     </row>
     <row r="43">
@@ -1127,7 +1127,7 @@
         <v>HIGH</v>
       </c>
       <c r="E43" t="str">
-        <v>0.139s</v>
+        <v>0.157s</v>
       </c>
     </row>
     <row r="44">
@@ -1144,7 +1144,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E44" t="str">
-        <v>0.146s</v>
+        <v>0.057s</v>
       </c>
     </row>
     <row r="45">
@@ -1161,7 +1161,7 @@
         <v>LOW</v>
       </c>
       <c r="E45" t="str">
-        <v>0.098s</v>
+        <v>0.145s</v>
       </c>
     </row>
     <row r="46">
@@ -1178,7 +1178,7 @@
         <v>HIGH</v>
       </c>
       <c r="E46" t="str">
-        <v>0.089s</v>
+        <v>0.149s</v>
       </c>
     </row>
     <row r="47">
@@ -1195,7 +1195,7 @@
         <v>LOW</v>
       </c>
       <c r="E47" t="str">
-        <v>0.089s</v>
+        <v>0.103s</v>
       </c>
     </row>
     <row r="48">
@@ -1212,7 +1212,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E48" t="str">
-        <v>0.077s</v>
+        <v>0.082s</v>
       </c>
     </row>
     <row r="49">
@@ -1229,7 +1229,7 @@
         <v>HIGH</v>
       </c>
       <c r="E49" t="str">
-        <v>0.138s</v>
+        <v>0.117s</v>
       </c>
     </row>
     <row r="50">
@@ -1246,7 +1246,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E50" t="str">
-        <v>0.062s</v>
+        <v>0.131s</v>
       </c>
     </row>
     <row r="51">
@@ -1263,7 +1263,7 @@
         <v>LOW</v>
       </c>
       <c r="E51" t="str">
-        <v>0.105s</v>
+        <v>0.092s</v>
       </c>
     </row>
     <row r="52">
@@ -1280,7 +1280,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E52" t="str">
-        <v>0.078s</v>
+        <v>0.139s</v>
       </c>
     </row>
     <row r="53">
@@ -1297,7 +1297,7 @@
         <v>LOW</v>
       </c>
       <c r="E53" t="str">
-        <v>0.061s</v>
+        <v>0.057s</v>
       </c>
     </row>
     <row r="54">
@@ -1314,7 +1314,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E54" t="str">
-        <v>0.139s</v>
+        <v>0.152s</v>
       </c>
     </row>
     <row r="55">
@@ -1331,7 +1331,7 @@
         <v>HIGH</v>
       </c>
       <c r="E55" t="str">
-        <v>0.060s</v>
+        <v>0.062s</v>
       </c>
     </row>
     <row r="56">
@@ -1348,7 +1348,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E56" t="str">
-        <v>0.066s</v>
+        <v>0.142s</v>
       </c>
     </row>
     <row r="57">
@@ -1365,7 +1365,7 @@
         <v>LOW</v>
       </c>
       <c r="E57" t="str">
-        <v>0.092s</v>
+        <v>0.130s</v>
       </c>
     </row>
     <row r="58">
@@ -1382,7 +1382,7 @@
         <v>HIGH</v>
       </c>
       <c r="E58" t="str">
-        <v>0.117s</v>
+        <v>0.041s</v>
       </c>
     </row>
     <row r="59">
@@ -1399,7 +1399,7 @@
         <v>LOW</v>
       </c>
       <c r="E59" t="str">
-        <v>0.157s</v>
+        <v>0.129s</v>
       </c>
     </row>
     <row r="60">
@@ -1416,7 +1416,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E60" t="str">
-        <v>0.130s</v>
+        <v>0.133s</v>
       </c>
     </row>
     <row r="61">
@@ -1433,7 +1433,7 @@
         <v>HIGH</v>
       </c>
       <c r="E61" t="str">
-        <v>0.115s</v>
+        <v>0.063s</v>
       </c>
     </row>
     <row r="62">
@@ -1450,7 +1450,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E62" t="str">
-        <v>0.118s</v>
+        <v>0.122s</v>
       </c>
     </row>
     <row r="63">
@@ -1467,7 +1467,7 @@
         <v>LOW</v>
       </c>
       <c r="E63" t="str">
-        <v>0.089s</v>
+        <v>0.094s</v>
       </c>
     </row>
     <row r="64">
@@ -1484,7 +1484,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E64" t="str">
-        <v>0.063s</v>
+        <v>0.147s</v>
       </c>
     </row>
     <row r="65">
@@ -1501,7 +1501,7 @@
         <v>LOW</v>
       </c>
       <c r="E65" t="str">
-        <v>0.134s</v>
+        <v>0.046s</v>
       </c>
     </row>
     <row r="66">
@@ -1518,7 +1518,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E66" t="str">
-        <v>0.045s</v>
+        <v>0.062s</v>
       </c>
     </row>
     <row r="67">
@@ -1535,7 +1535,7 @@
         <v>HIGH</v>
       </c>
       <c r="E67" t="str">
-        <v>0.052s</v>
+        <v>0.155s</v>
       </c>
     </row>
     <row r="68">
@@ -1552,7 +1552,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E68" t="str">
-        <v>0.047s</v>
+        <v>0.065s</v>
       </c>
     </row>
     <row r="69">
@@ -1569,7 +1569,7 @@
         <v>LOW</v>
       </c>
       <c r="E69" t="str">
-        <v>0.138s</v>
+        <v>0.083s</v>
       </c>
     </row>
     <row r="70">
@@ -1586,7 +1586,7 @@
         <v>HIGH</v>
       </c>
       <c r="E70" t="str">
-        <v>0.062s</v>
+        <v>0.121s</v>
       </c>
     </row>
     <row r="71">
@@ -1603,7 +1603,7 @@
         <v>LOW</v>
       </c>
       <c r="E71" t="str">
-        <v>0.072s</v>
+        <v>0.073s</v>
       </c>
     </row>
     <row r="72">
@@ -1620,7 +1620,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E72" t="str">
-        <v>0.116s</v>
+        <v>0.049s</v>
       </c>
     </row>
     <row r="73">
@@ -1637,7 +1637,7 @@
         <v>HIGH</v>
       </c>
       <c r="E73" t="str">
-        <v>0.071s</v>
+        <v>0.098s</v>
       </c>
     </row>
     <row r="74">
@@ -1654,7 +1654,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E74" t="str">
-        <v>0.051s</v>
+        <v>0.132s</v>
       </c>
     </row>
     <row r="75">
@@ -1671,7 +1671,7 @@
         <v>LOW</v>
       </c>
       <c r="E75" t="str">
-        <v>0.080s</v>
+        <v>0.139s</v>
       </c>
     </row>
     <row r="76">
@@ -1688,7 +1688,7 @@
         <v>HIGH</v>
       </c>
       <c r="E76" t="str">
-        <v>0.114s</v>
+        <v>0.112s</v>
       </c>
     </row>
     <row r="77">
@@ -1705,7 +1705,7 @@
         <v>LOW</v>
       </c>
       <c r="E77" t="str">
-        <v>0.121s</v>
+        <v>0.076s</v>
       </c>
     </row>
     <row r="78">
@@ -1722,7 +1722,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E78" t="str">
-        <v>0.072s</v>
+        <v>0.155s</v>
       </c>
     </row>
     <row r="79">
@@ -1739,7 +1739,7 @@
         <v>HIGH</v>
       </c>
       <c r="E79" t="str">
-        <v>0.077s</v>
+        <v>0.083s</v>
       </c>
     </row>
     <row r="80">
@@ -1756,7 +1756,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E80" t="str">
-        <v>0.155s</v>
+        <v>0.078s</v>
       </c>
     </row>
     <row r="81">
@@ -1773,7 +1773,7 @@
         <v>LOW</v>
       </c>
       <c r="E81" t="str">
-        <v>0.108s</v>
+        <v>0.052s</v>
       </c>
     </row>
     <row r="82">
@@ -1790,7 +1790,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E82" t="str">
-        <v>0.124s</v>
+        <v>0.150s</v>
       </c>
     </row>
     <row r="83">
@@ -1807,7 +1807,7 @@
         <v>LOW</v>
       </c>
       <c r="E83" t="str">
-        <v>0.047s</v>
+        <v>0.086s</v>
       </c>
     </row>
     <row r="84">
@@ -1824,7 +1824,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E84" t="str">
-        <v>0.121s</v>
+        <v>0.093s</v>
       </c>
     </row>
     <row r="85">
@@ -1841,7 +1841,7 @@
         <v>HIGH</v>
       </c>
       <c r="E85" t="str">
-        <v>0.051s</v>
+        <v>0.147s</v>
       </c>
     </row>
     <row r="86">
@@ -1858,7 +1858,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E86" t="str">
-        <v>0.055s</v>
+        <v>0.057s</v>
       </c>
     </row>
     <row r="87">
@@ -1875,7 +1875,7 @@
         <v>LOW</v>
       </c>
       <c r="E87" t="str">
-        <v>0.148s</v>
+        <v>0.055s</v>
       </c>
     </row>
     <row r="88">
@@ -1892,7 +1892,7 @@
         <v>HIGH</v>
       </c>
       <c r="E88" t="str">
-        <v>0.088s</v>
+        <v>0.055s</v>
       </c>
     </row>
     <row r="89">
@@ -1909,7 +1909,7 @@
         <v>LOW</v>
       </c>
       <c r="E89" t="str">
-        <v>0.138s</v>
+        <v>0.148s</v>
       </c>
     </row>
     <row r="90">
@@ -1926,7 +1926,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E90" t="str">
-        <v>0.156s</v>
+        <v>0.068s</v>
       </c>
     </row>
     <row r="91">
@@ -1943,7 +1943,7 @@
         <v>LOW</v>
       </c>
       <c r="E91" t="str">
-        <v>0.127s</v>
+        <v>0.138s</v>
       </c>
     </row>
     <row r="92">
@@ -1960,7 +1960,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E92" t="str">
-        <v>0.139s</v>
+        <v>0.071s</v>
       </c>
     </row>
     <row r="93">
@@ -1977,7 +1977,7 @@
         <v>HIGH</v>
       </c>
       <c r="E93" t="str">
-        <v>0.160s</v>
+        <v>0.048s</v>
       </c>
     </row>
     <row r="94">
@@ -1994,7 +1994,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E94" t="str">
-        <v>0.043s</v>
+        <v>0.142s</v>
       </c>
     </row>
     <row r="95">
@@ -2011,7 +2011,7 @@
         <v>LOW</v>
       </c>
       <c r="E95" t="str">
-        <v>0.145s</v>
+        <v>0.087s</v>
       </c>
     </row>
     <row r="96">
@@ -2028,7 +2028,7 @@
         <v>HIGH</v>
       </c>
       <c r="E96" t="str">
-        <v>0.091s</v>
+        <v>0.058s</v>
       </c>
     </row>
     <row r="97">
@@ -2045,7 +2045,7 @@
         <v>LOW</v>
       </c>
       <c r="E97" t="str">
-        <v>0.071s</v>
+        <v>0.104s</v>
       </c>
     </row>
     <row r="98">
@@ -2062,7 +2062,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E98" t="str">
-        <v>0.077s</v>
+        <v>0.089s</v>
       </c>
     </row>
     <row r="99">
@@ -2079,7 +2079,7 @@
         <v>HIGH</v>
       </c>
       <c r="E99" t="str">
-        <v>0.144s</v>
+        <v>0.103s</v>
       </c>
     </row>
     <row r="100">
@@ -2096,7 +2096,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E100" t="str">
-        <v>0.065s</v>
+        <v>0.139s</v>
       </c>
     </row>
     <row r="101">
@@ -2113,7 +2113,7 @@
         <v>LOW</v>
       </c>
       <c r="E101" t="str">
-        <v>0.080s</v>
+        <v>0.081s</v>
       </c>
     </row>
     <row r="102">
@@ -2130,7 +2130,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E102" t="str">
-        <v>0.148s</v>
+        <v>0.054s</v>
       </c>
     </row>
     <row r="103">
@@ -2147,7 +2147,7 @@
         <v>LOW</v>
       </c>
       <c r="E103" t="str">
-        <v>0.114s</v>
+        <v>0.120s</v>
       </c>
     </row>
     <row r="104">
@@ -2164,7 +2164,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E104" t="str">
-        <v>0.155s</v>
+        <v>0.071s</v>
       </c>
     </row>
     <row r="105">
@@ -2181,7 +2181,7 @@
         <v>HIGH</v>
       </c>
       <c r="E105" t="str">
-        <v>0.096s</v>
+        <v>0.102s</v>
       </c>
     </row>
     <row r="106">
@@ -2198,7 +2198,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E106" t="str">
-        <v>0.044s</v>
+        <v>0.086s</v>
       </c>
     </row>
     <row r="107">
@@ -2215,7 +2215,7 @@
         <v>LOW</v>
       </c>
       <c r="E107" t="str">
-        <v>0.151s</v>
+        <v>0.078s</v>
       </c>
     </row>
     <row r="108">
@@ -2232,7 +2232,7 @@
         <v>HIGH</v>
       </c>
       <c r="E108" t="str">
-        <v>0.125s</v>
+        <v>0.137s</v>
       </c>
     </row>
     <row r="109">
@@ -2249,7 +2249,7 @@
         <v>LOW</v>
       </c>
       <c r="E109" t="str">
-        <v>0.070s</v>
+        <v>0.062s</v>
       </c>
     </row>
     <row r="110">
@@ -2266,7 +2266,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E110" t="str">
-        <v>0.152s</v>
+        <v>0.055s</v>
       </c>
     </row>
     <row r="111">
@@ -2283,7 +2283,7 @@
         <v>LOW</v>
       </c>
       <c r="E111" t="str">
-        <v>0.121s</v>
+        <v>0.109s</v>
       </c>
     </row>
     <row r="112">
@@ -2300,7 +2300,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E112" t="str">
-        <v>0.086s</v>
+        <v>0.097s</v>
       </c>
     </row>
     <row r="113">
@@ -2317,7 +2317,7 @@
         <v>HIGH</v>
       </c>
       <c r="E113" t="str">
-        <v>0.080s</v>
+        <v>0.108s</v>
       </c>
     </row>
     <row r="114">
@@ -2334,7 +2334,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E114" t="str">
-        <v>0.072s</v>
+        <v>0.111s</v>
       </c>
     </row>
     <row r="115">
@@ -2351,7 +2351,7 @@
         <v>LOW</v>
       </c>
       <c r="E115" t="str">
-        <v>0.086s</v>
+        <v>0.150s</v>
       </c>
     </row>
     <row r="116">
@@ -2368,7 +2368,7 @@
         <v>HIGH</v>
       </c>
       <c r="E116" t="str">
-        <v>0.143s</v>
+        <v>0.136s</v>
       </c>
     </row>
     <row r="117">
@@ -2385,7 +2385,7 @@
         <v>LOW</v>
       </c>
       <c r="E117" t="str">
-        <v>0.155s</v>
+        <v>0.149s</v>
       </c>
     </row>
     <row r="118">
@@ -2402,7 +2402,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E118" t="str">
-        <v>0.108s</v>
+        <v>0.076s</v>
       </c>
     </row>
     <row r="119">
@@ -2419,7 +2419,7 @@
         <v>HIGH</v>
       </c>
       <c r="E119" t="str">
-        <v>0.115s</v>
+        <v>0.065s</v>
       </c>
     </row>
     <row r="120">
@@ -2436,7 +2436,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E120" t="str">
-        <v>0.044s</v>
+        <v>0.139s</v>
       </c>
     </row>
     <row r="121">
@@ -2453,7 +2453,7 @@
         <v>LOW</v>
       </c>
       <c r="E121" t="str">
-        <v>0.114s</v>
+        <v>0.147s</v>
       </c>
     </row>
     <row r="122">
@@ -2470,7 +2470,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E122" t="str">
-        <v>0.093s</v>
+        <v>0.121s</v>
       </c>
     </row>
     <row r="123">
@@ -2487,7 +2487,7 @@
         <v>LOW</v>
       </c>
       <c r="E123" t="str">
-        <v>0.130s</v>
+        <v>0.058s</v>
       </c>
     </row>
     <row r="124">
@@ -2504,7 +2504,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E124" t="str">
-        <v>0.113s</v>
+        <v>0.069s</v>
       </c>
     </row>
     <row r="125">
@@ -2521,7 +2521,7 @@
         <v>HIGH</v>
       </c>
       <c r="E125" t="str">
-        <v>0.115s</v>
+        <v>0.040s</v>
       </c>
     </row>
     <row r="126">
@@ -2538,7 +2538,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E126" t="str">
-        <v>0.080s</v>
+        <v>0.138s</v>
       </c>
     </row>
     <row r="127">
@@ -2555,7 +2555,7 @@
         <v>LOW</v>
       </c>
       <c r="E127" t="str">
-        <v>0.136s</v>
+        <v>0.132s</v>
       </c>
     </row>
     <row r="128">
@@ -2572,7 +2572,7 @@
         <v>HIGH</v>
       </c>
       <c r="E128" t="str">
-        <v>0.157s</v>
+        <v>0.092s</v>
       </c>
     </row>
     <row r="129">
@@ -2589,7 +2589,7 @@
         <v>LOW</v>
       </c>
       <c r="E129" t="str">
-        <v>0.072s</v>
+        <v>0.135s</v>
       </c>
     </row>
     <row r="130">
@@ -2606,7 +2606,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E130" t="str">
-        <v>0.121s</v>
+        <v>0.090s</v>
       </c>
     </row>
     <row r="131">
@@ -2640,7 +2640,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E132" t="str">
-        <v>0.149s</v>
+        <v>0.082s</v>
       </c>
     </row>
     <row r="133">
@@ -2657,7 +2657,7 @@
         <v>LOW</v>
       </c>
       <c r="E133" t="str">
-        <v>0.093s</v>
+        <v>0.114s</v>
       </c>
     </row>
     <row r="134">
@@ -2674,7 +2674,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E134" t="str">
-        <v>0.043s</v>
+        <v>0.065s</v>
       </c>
     </row>
     <row r="135">
@@ -2691,7 +2691,7 @@
         <v>LOW</v>
       </c>
       <c r="E135" t="str">
-        <v>0.077s</v>
+        <v>0.055s</v>
       </c>
     </row>
     <row r="136">
@@ -2708,7 +2708,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E136" t="str">
-        <v>0.056s</v>
+        <v>0.100s</v>
       </c>
     </row>
     <row r="137">
@@ -2725,7 +2725,7 @@
         <v>HIGH</v>
       </c>
       <c r="E137" t="str">
-        <v>0.050s</v>
+        <v>0.127s</v>
       </c>
     </row>
     <row r="138">
@@ -2742,7 +2742,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E138" t="str">
-        <v>0.153s</v>
+        <v>0.139s</v>
       </c>
     </row>
     <row r="139">
@@ -2759,7 +2759,7 @@
         <v>LOW</v>
       </c>
       <c r="E139" t="str">
-        <v>0.054s</v>
+        <v>0.052s</v>
       </c>
     </row>
     <row r="140">
@@ -2776,7 +2776,7 @@
         <v>HIGH</v>
       </c>
       <c r="E140" t="str">
-        <v>0.153s</v>
+        <v>0.148s</v>
       </c>
     </row>
     <row r="141">
@@ -2793,7 +2793,7 @@
         <v>LOW</v>
       </c>
       <c r="E141" t="str">
-        <v>0.097s</v>
+        <v>0.063s</v>
       </c>
     </row>
     <row r="142">
@@ -2810,7 +2810,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E142" t="str">
-        <v>0.117s</v>
+        <v>0.157s</v>
       </c>
     </row>
     <row r="143">
@@ -2827,7 +2827,7 @@
         <v>HIGH</v>
       </c>
       <c r="E143" t="str">
-        <v>0.099s</v>
+        <v>0.123s</v>
       </c>
     </row>
     <row r="144">
@@ -2844,7 +2844,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E144" t="str">
-        <v>0.085s</v>
+        <v>0.126s</v>
       </c>
     </row>
     <row r="145">
@@ -2861,7 +2861,7 @@
         <v>LOW</v>
       </c>
       <c r="E145" t="str">
-        <v>0.114s</v>
+        <v>0.089s</v>
       </c>
     </row>
     <row r="146">
@@ -2878,7 +2878,7 @@
         <v>HIGH</v>
       </c>
       <c r="E146" t="str">
-        <v>0.151s</v>
+        <v>0.123s</v>
       </c>
     </row>
     <row r="147">
@@ -2895,7 +2895,7 @@
         <v>LOW</v>
       </c>
       <c r="E147" t="str">
-        <v>0.067s</v>
+        <v>0.058s</v>
       </c>
     </row>
     <row r="148">
@@ -2912,7 +2912,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E148" t="str">
-        <v>0.066s</v>
+        <v>0.109s</v>
       </c>
     </row>
     <row r="149">
@@ -2929,7 +2929,7 @@
         <v>HIGH</v>
       </c>
       <c r="E149" t="str">
-        <v>0.111s</v>
+        <v>0.152s</v>
       </c>
     </row>
     <row r="150">
@@ -2946,7 +2946,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E150" t="str">
-        <v>0.133s</v>
+        <v>0.130s</v>
       </c>
     </row>
     <row r="151">
@@ -2963,7 +2963,7 @@
         <v>LOW</v>
       </c>
       <c r="E151" t="str">
-        <v>0.093s</v>
+        <v>0.142s</v>
       </c>
     </row>
     <row r="152">
@@ -2980,7 +2980,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E152" t="str">
-        <v>0.101s</v>
+        <v>0.102s</v>
       </c>
     </row>
     <row r="153">
@@ -2997,7 +2997,7 @@
         <v>LOW</v>
       </c>
       <c r="E153" t="str">
-        <v>0.105s</v>
+        <v>0.159s</v>
       </c>
     </row>
     <row r="154">
@@ -3014,7 +3014,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E154" t="str">
-        <v>0.048s</v>
+        <v>0.044s</v>
       </c>
     </row>
     <row r="155">
@@ -3031,7 +3031,7 @@
         <v>HIGH</v>
       </c>
       <c r="E155" t="str">
-        <v>0.125s</v>
+        <v>0.108s</v>
       </c>
     </row>
     <row r="156">
@@ -3048,7 +3048,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E156" t="str">
-        <v>0.043s</v>
+        <v>0.109s</v>
       </c>
     </row>
     <row r="157">
@@ -3065,7 +3065,7 @@
         <v>LOW</v>
       </c>
       <c r="E157" t="str">
-        <v>0.138s</v>
+        <v>0.076s</v>
       </c>
     </row>
     <row r="158">
@@ -3082,7 +3082,7 @@
         <v>HIGH</v>
       </c>
       <c r="E158" t="str">
-        <v>0.103s</v>
+        <v>0.134s</v>
       </c>
     </row>
     <row r="159">
@@ -3099,7 +3099,7 @@
         <v>LOW</v>
       </c>
       <c r="E159" t="str">
-        <v>0.132s</v>
+        <v>0.067s</v>
       </c>
     </row>
     <row r="160">
@@ -3116,7 +3116,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E160" t="str">
-        <v>0.148s</v>
+        <v>0.113s</v>
       </c>
     </row>
     <row r="161">
@@ -3133,7 +3133,7 @@
         <v>LOW</v>
       </c>
       <c r="E161" t="str">
-        <v>0.113s</v>
+        <v>0.099s</v>
       </c>
     </row>
     <row r="162">
@@ -3150,7 +3150,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E162" t="str">
-        <v>0.104s</v>
+        <v>0.119s</v>
       </c>
     </row>
     <row r="163">
@@ -3167,7 +3167,7 @@
         <v>HIGH</v>
       </c>
       <c r="E163" t="str">
-        <v>0.124s</v>
+        <v>0.053s</v>
       </c>
     </row>
     <row r="164">
@@ -3184,7 +3184,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E164" t="str">
-        <v>0.066s</v>
+        <v>0.103s</v>
       </c>
     </row>
     <row r="165">
@@ -3201,7 +3201,7 @@
         <v>LOW</v>
       </c>
       <c r="E165" t="str">
-        <v>0.130s</v>
+        <v>0.085s</v>
       </c>
     </row>
     <row r="166">
@@ -3218,7 +3218,7 @@
         <v>HIGH</v>
       </c>
       <c r="E166" t="str">
-        <v>0.051s</v>
+        <v>0.129s</v>
       </c>
     </row>
     <row r="167">
@@ -3235,7 +3235,7 @@
         <v>LOW</v>
       </c>
       <c r="E167" t="str">
-        <v>0.126s</v>
+        <v>0.082s</v>
       </c>
     </row>
     <row r="168">
@@ -3252,7 +3252,7 @@
         <v>HIGH</v>
       </c>
       <c r="E168" t="str">
-        <v>0.066s</v>
+        <v>0.048s</v>
       </c>
     </row>
     <row r="169">
@@ -3269,7 +3269,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E169" t="str">
-        <v>0.134s</v>
+        <v>0.058s</v>
       </c>
     </row>
     <row r="170">
@@ -3286,7 +3286,7 @@
         <v>LOW</v>
       </c>
       <c r="E170" t="str">
-        <v>0.098s</v>
+        <v>0.124s</v>
       </c>
     </row>
     <row r="171">
@@ -3303,7 +3303,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E171" t="str">
-        <v>0.081s</v>
+        <v>0.152s</v>
       </c>
     </row>
     <row r="172">
@@ -3320,7 +3320,7 @@
         <v>LOW</v>
       </c>
       <c r="E172" t="str">
-        <v>0.137s</v>
+        <v>0.128s</v>
       </c>
     </row>
     <row r="173">
@@ -3337,7 +3337,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E173" t="str">
-        <v>0.146s</v>
+        <v>0.125s</v>
       </c>
     </row>
     <row r="174">
@@ -3354,7 +3354,7 @@
         <v>HIGH</v>
       </c>
       <c r="E174" t="str">
-        <v>0.117s</v>
+        <v>0.146s</v>
       </c>
     </row>
     <row r="175">
@@ -3371,7 +3371,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E175" t="str">
-        <v>0.117s</v>
+        <v>0.125s</v>
       </c>
     </row>
     <row r="176">
@@ -3388,7 +3388,7 @@
         <v>LOW</v>
       </c>
       <c r="E176" t="str">
-        <v>0.056s</v>
+        <v>0.122s</v>
       </c>
     </row>
     <row r="177">
@@ -3405,7 +3405,7 @@
         <v>HIGH</v>
       </c>
       <c r="E177" t="str">
-        <v>0.097s</v>
+        <v>0.159s</v>
       </c>
     </row>
     <row r="178">
@@ -3422,7 +3422,7 @@
         <v>LOW</v>
       </c>
       <c r="E178" t="str">
-        <v>0.117s</v>
+        <v>0.053s</v>
       </c>
     </row>
     <row r="179">
@@ -3439,7 +3439,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E179" t="str">
-        <v>0.042s</v>
+        <v>0.113s</v>
       </c>
     </row>
     <row r="180">
@@ -3456,7 +3456,7 @@
         <v>HIGH</v>
       </c>
       <c r="E180" t="str">
-        <v>0.051s</v>
+        <v>0.111s</v>
       </c>
     </row>
     <row r="181">
@@ -3473,7 +3473,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E181" t="str">
-        <v>0.135s</v>
+        <v>0.117s</v>
       </c>
     </row>
     <row r="182">
@@ -3490,7 +3490,7 @@
         <v>LOW</v>
       </c>
       <c r="E182" t="str">
-        <v>0.113s</v>
+        <v>0.078s</v>
       </c>
     </row>
     <row r="183">
@@ -3507,7 +3507,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E183" t="str">
-        <v>0.057s</v>
+        <v>0.090s</v>
       </c>
     </row>
     <row r="184">
@@ -3524,7 +3524,7 @@
         <v>LOW</v>
       </c>
       <c r="E184" t="str">
-        <v>0.080s</v>
+        <v>0.158s</v>
       </c>
     </row>
     <row r="185">
@@ -3541,7 +3541,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E185" t="str">
-        <v>0.131s</v>
+        <v>0.141s</v>
       </c>
     </row>
     <row r="186">
@@ -3558,7 +3558,7 @@
         <v>HIGH</v>
       </c>
       <c r="E186" t="str">
-        <v>0.159s</v>
+        <v>0.139s</v>
       </c>
     </row>
     <row r="187">
@@ -3575,7 +3575,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E187" t="str">
-        <v>0.143s</v>
+        <v>0.092s</v>
       </c>
     </row>
     <row r="188">
@@ -3592,7 +3592,7 @@
         <v>LOW</v>
       </c>
       <c r="E188" t="str">
-        <v>0.117s</v>
+        <v>0.044s</v>
       </c>
     </row>
     <row r="189">
@@ -3609,7 +3609,7 @@
         <v>HIGH</v>
       </c>
       <c r="E189" t="str">
-        <v>0.149s</v>
+        <v>0.135s</v>
       </c>
     </row>
     <row r="190">
@@ -3626,7 +3626,7 @@
         <v>LOW</v>
       </c>
       <c r="E190" t="str">
-        <v>0.147s</v>
+        <v>0.064s</v>
       </c>
     </row>
     <row r="191">
@@ -3643,7 +3643,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E191" t="str">
-        <v>0.062s</v>
+        <v>0.141s</v>
       </c>
     </row>
     <row r="192">
@@ -3660,7 +3660,7 @@
         <v>HIGH</v>
       </c>
       <c r="E192" t="str">
-        <v>0.074s</v>
+        <v>0.051s</v>
       </c>
     </row>
     <row r="193">
@@ -3677,7 +3677,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E193" t="str">
-        <v>0.103s</v>
+        <v>0.156s</v>
       </c>
     </row>
     <row r="194">
@@ -3694,7 +3694,7 @@
         <v>LOW</v>
       </c>
       <c r="E194" t="str">
-        <v>0.147s</v>
+        <v>0.158s</v>
       </c>
     </row>
     <row r="195">
@@ -3711,7 +3711,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E195" t="str">
-        <v>0.136s</v>
+        <v>0.143s</v>
       </c>
     </row>
     <row r="196">
@@ -3728,7 +3728,7 @@
         <v>LOW</v>
       </c>
       <c r="E196" t="str">
-        <v>0.098s</v>
+        <v>0.120s</v>
       </c>
     </row>
     <row r="197">
@@ -3745,7 +3745,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E197" t="str">
-        <v>0.085s</v>
+        <v>0.048s</v>
       </c>
     </row>
     <row r="198">
@@ -3762,7 +3762,7 @@
         <v>HIGH</v>
       </c>
       <c r="E198" t="str">
-        <v>0.123s</v>
+        <v>0.102s</v>
       </c>
     </row>
     <row r="199">
@@ -3779,7 +3779,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E199" t="str">
-        <v>0.122s</v>
+        <v>0.106s</v>
       </c>
     </row>
     <row r="200">
@@ -3796,7 +3796,7 @@
         <v>LOW</v>
       </c>
       <c r="E200" t="str">
-        <v>0.058s</v>
+        <v>0.077s</v>
       </c>
     </row>
     <row r="201">
@@ -3813,7 +3813,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E201" t="str">
-        <v>0.065s</v>
+        <v>0.107s</v>
       </c>
     </row>
     <row r="202">
@@ -3830,7 +3830,7 @@
         <v>HIGH</v>
       </c>
       <c r="E202" t="str">
-        <v>0.066s</v>
+        <v>0.125s</v>
       </c>
     </row>
     <row r="203">
@@ -3847,7 +3847,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E203" t="str">
-        <v>0.055s</v>
+        <v>0.126s</v>
       </c>
     </row>
     <row r="204">
@@ -3864,7 +3864,7 @@
         <v>LOW</v>
       </c>
       <c r="E204" t="str">
-        <v>0.150s</v>
+        <v>0.078s</v>
       </c>
     </row>
     <row r="205">
@@ -3881,7 +3881,7 @@
         <v>HIGH</v>
       </c>
       <c r="E205" t="str">
-        <v>0.042s</v>
+        <v>0.155s</v>
       </c>
     </row>
     <row r="206">
@@ -3898,7 +3898,7 @@
         <v>LOW</v>
       </c>
       <c r="E206" t="str">
-        <v>0.112s</v>
+        <v>0.081s</v>
       </c>
     </row>
     <row r="207">
@@ -3915,7 +3915,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E207" t="str">
-        <v>0.090s</v>
+        <v>0.051s</v>
       </c>
     </row>
     <row r="208">
@@ -3932,7 +3932,7 @@
         <v>HIGH</v>
       </c>
       <c r="E208" t="str">
-        <v>0.158s</v>
+        <v>0.134s</v>
       </c>
     </row>
     <row r="209">
@@ -3949,7 +3949,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E209" t="str">
-        <v>0.122s</v>
+        <v>0.144s</v>
       </c>
     </row>
     <row r="210">
@@ -3966,7 +3966,7 @@
         <v>LOW</v>
       </c>
       <c r="E210" t="str">
-        <v>0.066s</v>
+        <v>0.077s</v>
       </c>
     </row>
     <row r="211">
@@ -3983,7 +3983,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E211" t="str">
-        <v>0.149s</v>
+        <v>0.117s</v>
       </c>
     </row>
     <row r="212">
@@ -4000,7 +4000,7 @@
         <v>LOW</v>
       </c>
       <c r="E212" t="str">
-        <v>0.111s</v>
+        <v>0.145s</v>
       </c>
     </row>
     <row r="213">
@@ -4017,7 +4017,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E213" t="str">
-        <v>0.052s</v>
+        <v>0.108s</v>
       </c>
     </row>
     <row r="214">
@@ -4034,7 +4034,7 @@
         <v>HIGH</v>
       </c>
       <c r="E214" t="str">
-        <v>0.062s</v>
+        <v>0.086s</v>
       </c>
     </row>
     <row r="215">
@@ -4051,7 +4051,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E215" t="str">
-        <v>0.128s</v>
+        <v>0.065s</v>
       </c>
     </row>
     <row r="216">
@@ -4068,7 +4068,7 @@
         <v>LOW</v>
       </c>
       <c r="E216" t="str">
-        <v>0.130s</v>
+        <v>0.149s</v>
       </c>
     </row>
     <row r="217">
@@ -4085,7 +4085,7 @@
         <v>HIGH</v>
       </c>
       <c r="E217" t="str">
-        <v>0.063s</v>
+        <v>0.082s</v>
       </c>
     </row>
     <row r="218">
@@ -4102,7 +4102,7 @@
         <v>LOW</v>
       </c>
       <c r="E218" t="str">
-        <v>0.127s</v>
+        <v>0.088s</v>
       </c>
     </row>
     <row r="219">
@@ -4119,7 +4119,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E219" t="str">
-        <v>0.102s</v>
+        <v>0.050s</v>
       </c>
     </row>
     <row r="220">
@@ -4136,7 +4136,7 @@
         <v>HIGH</v>
       </c>
       <c r="E220" t="str">
-        <v>0.113s</v>
+        <v>0.089s</v>
       </c>
     </row>
     <row r="221">
@@ -4153,7 +4153,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E221" t="str">
-        <v>0.132s</v>
+        <v>0.109s</v>
       </c>
     </row>
     <row r="222">
@@ -4170,7 +4170,7 @@
         <v>LOW</v>
       </c>
       <c r="E222" t="str">
-        <v>0.135s</v>
+        <v>0.068s</v>
       </c>
     </row>
     <row r="223">
@@ -4187,7 +4187,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E223" t="str">
-        <v>0.081s</v>
+        <v>0.117s</v>
       </c>
     </row>
     <row r="224">
@@ -4204,7 +4204,7 @@
         <v>LOW</v>
       </c>
       <c r="E224" t="str">
-        <v>0.124s</v>
+        <v>0.112s</v>
       </c>
     </row>
     <row r="225">
@@ -4221,7 +4221,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E225" t="str">
-        <v>0.071s</v>
+        <v>0.074s</v>
       </c>
     </row>
     <row r="226">
@@ -4238,7 +4238,7 @@
         <v>HIGH</v>
       </c>
       <c r="E226" t="str">
-        <v>0.063s</v>
+        <v>0.151s</v>
       </c>
     </row>
     <row r="227">
@@ -4255,7 +4255,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E227" t="str">
-        <v>0.133s</v>
+        <v>0.100s</v>
       </c>
     </row>
     <row r="228">
@@ -4272,7 +4272,7 @@
         <v>LOW</v>
       </c>
       <c r="E228" t="str">
-        <v>0.123s</v>
+        <v>0.047s</v>
       </c>
     </row>
     <row r="229">
@@ -4289,7 +4289,7 @@
         <v>HIGH</v>
       </c>
       <c r="E229" t="str">
-        <v>0.063s</v>
+        <v>0.067s</v>
       </c>
     </row>
     <row r="230">
@@ -4306,7 +4306,7 @@
         <v>LOW</v>
       </c>
       <c r="E230" t="str">
-        <v>0.051s</v>
+        <v>0.107s</v>
       </c>
     </row>
     <row r="231">
@@ -4323,7 +4323,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E231" t="str">
-        <v>0.070s</v>
+        <v>0.071s</v>
       </c>
     </row>
     <row r="232">
@@ -4340,7 +4340,7 @@
         <v>HIGH</v>
       </c>
       <c r="E232" t="str">
-        <v>0.079s</v>
+        <v>0.101s</v>
       </c>
     </row>
     <row r="233">
@@ -4357,7 +4357,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E233" t="str">
-        <v>0.148s</v>
+        <v>0.137s</v>
       </c>
     </row>
     <row r="234">
@@ -4374,7 +4374,7 @@
         <v>LOW</v>
       </c>
       <c r="E234" t="str">
-        <v>0.140s</v>
+        <v>0.079s</v>
       </c>
     </row>
     <row r="235">
@@ -4391,7 +4391,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E235" t="str">
-        <v>0.104s</v>
+        <v>0.096s</v>
       </c>
     </row>
     <row r="236">
@@ -4408,7 +4408,7 @@
         <v>LOW</v>
       </c>
       <c r="E236" t="str">
-        <v>0.145s</v>
+        <v>0.135s</v>
       </c>
     </row>
     <row r="237">
@@ -4425,7 +4425,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E237" t="str">
-        <v>0.106s</v>
+        <v>0.100s</v>
       </c>
     </row>
     <row r="238">
@@ -4442,7 +4442,7 @@
         <v>HIGH</v>
       </c>
       <c r="E238" t="str">
-        <v>0.126s</v>
+        <v>0.146s</v>
       </c>
     </row>
     <row r="239">
@@ -4459,7 +4459,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E239" t="str">
-        <v>0.110s</v>
+        <v>0.042s</v>
       </c>
     </row>
     <row r="240">
@@ -4476,7 +4476,7 @@
         <v>LOW</v>
       </c>
       <c r="E240" t="str">
-        <v>0.067s</v>
+        <v>0.063s</v>
       </c>
     </row>
     <row r="241">
@@ -4493,7 +4493,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E241" t="str">
-        <v>0.054s</v>
+        <v>0.152s</v>
       </c>
     </row>
     <row r="242">
@@ -4510,7 +4510,7 @@
         <v>HIGH</v>
       </c>
       <c r="E242" t="str">
-        <v>0.058s</v>
+        <v>0.147s</v>
       </c>
     </row>
     <row r="243">
@@ -4527,7 +4527,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E243" t="str">
-        <v>0.094s</v>
+        <v>0.040s</v>
       </c>
     </row>
     <row r="244">
@@ -4544,7 +4544,7 @@
         <v>LOW</v>
       </c>
       <c r="E244" t="str">
-        <v>0.110s</v>
+        <v>0.081s</v>
       </c>
     </row>
     <row r="245">
@@ -4561,7 +4561,7 @@
         <v>HIGH</v>
       </c>
       <c r="E245" t="str">
-        <v>0.124s</v>
+        <v>0.092s</v>
       </c>
     </row>
     <row r="246">
@@ -4578,7 +4578,7 @@
         <v>LOW</v>
       </c>
       <c r="E246" t="str">
-        <v>0.151s</v>
+        <v>0.143s</v>
       </c>
     </row>
     <row r="247">
@@ -4595,7 +4595,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E247" t="str">
-        <v>0.118s</v>
+        <v>0.064s</v>
       </c>
     </row>
     <row r="248">
@@ -4612,7 +4612,7 @@
         <v>HIGH</v>
       </c>
       <c r="E248" t="str">
-        <v>0.044s</v>
+        <v>0.075s</v>
       </c>
     </row>
     <row r="249">
@@ -4629,7 +4629,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E249" t="str">
-        <v>0.041s</v>
+        <v>0.138s</v>
       </c>
     </row>
     <row r="250">
@@ -4646,7 +4646,7 @@
         <v>LOW</v>
       </c>
       <c r="E250" t="str">
-        <v>0.143s</v>
+        <v>0.053s</v>
       </c>
     </row>
     <row r="251">
@@ -4663,7 +4663,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E251" t="str">
-        <v>0.070s</v>
+        <v>0.072s</v>
       </c>
     </row>
     <row r="252">
@@ -4680,7 +4680,7 @@
         <v>LOW</v>
       </c>
       <c r="E252" t="str">
-        <v>0.114s</v>
+        <v>0.137s</v>
       </c>
     </row>
     <row r="253">
@@ -4697,7 +4697,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E253" t="str">
-        <v>0.049s</v>
+        <v>0.071s</v>
       </c>
     </row>
     <row r="254">
@@ -4714,7 +4714,7 @@
         <v>HIGH</v>
       </c>
       <c r="E254" t="str">
-        <v>0.108s</v>
+        <v>0.148s</v>
       </c>
     </row>
     <row r="255">
@@ -4731,7 +4731,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E255" t="str">
-        <v>0.155s</v>
+        <v>0.147s</v>
       </c>
     </row>
     <row r="256">
@@ -4748,7 +4748,7 @@
         <v>LOW</v>
       </c>
       <c r="E256" t="str">
-        <v>0.081s</v>
+        <v>0.103s</v>
       </c>
     </row>
     <row r="257">
@@ -4765,7 +4765,7 @@
         <v>HIGH</v>
       </c>
       <c r="E257" t="str">
-        <v>0.123s</v>
+        <v>0.096s</v>
       </c>
     </row>
     <row r="258">
@@ -4782,7 +4782,7 @@
         <v>LOW</v>
       </c>
       <c r="E258" t="str">
-        <v>0.097s</v>
+        <v>0.057s</v>
       </c>
     </row>
     <row r="259">
@@ -4816,7 +4816,7 @@
         <v>LOW</v>
       </c>
       <c r="E260" t="str">
-        <v>0.049s</v>
+        <v>0.051s</v>
       </c>
     </row>
     <row r="261">
@@ -4833,7 +4833,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E261" t="str">
-        <v>0.072s</v>
+        <v>0.150s</v>
       </c>
     </row>
     <row r="262">
@@ -4850,7 +4850,7 @@
         <v>HIGH</v>
       </c>
       <c r="E262" t="str">
-        <v>0.086s</v>
+        <v>0.041s</v>
       </c>
     </row>
     <row r="263">
@@ -4867,7 +4867,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E263" t="str">
-        <v>0.111s</v>
+        <v>0.045s</v>
       </c>
     </row>
     <row r="264">
@@ -4884,7 +4884,7 @@
         <v>LOW</v>
       </c>
       <c r="E264" t="str">
-        <v>0.075s</v>
+        <v>0.125s</v>
       </c>
     </row>
     <row r="265">
@@ -4901,7 +4901,7 @@
         <v>HIGH</v>
       </c>
       <c r="E265" t="str">
-        <v>0.080s</v>
+        <v>0.148s</v>
       </c>
     </row>
     <row r="266">
@@ -4918,7 +4918,7 @@
         <v>LOW</v>
       </c>
       <c r="E266" t="str">
-        <v>0.076s</v>
+        <v>0.055s</v>
       </c>
     </row>
     <row r="267">
@@ -4935,7 +4935,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E267" t="str">
-        <v>0.070s</v>
+        <v>0.079s</v>
       </c>
     </row>
     <row r="268">
@@ -4952,7 +4952,7 @@
         <v>HIGH</v>
       </c>
       <c r="E268" t="str">
-        <v>0.049s</v>
+        <v>0.044s</v>
       </c>
     </row>
     <row r="269">
@@ -4969,7 +4969,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E269" t="str">
-        <v>0.158s</v>
+        <v>0.057s</v>
       </c>
     </row>
     <row r="270">
@@ -4986,7 +4986,7 @@
         <v>LOW</v>
       </c>
       <c r="E270" t="str">
-        <v>0.067s</v>
+        <v>0.096s</v>
       </c>
     </row>
     <row r="271">
@@ -5003,7 +5003,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E271" t="str">
-        <v>0.059s</v>
+        <v>0.040s</v>
       </c>
     </row>
     <row r="272">
@@ -5037,7 +5037,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E273" t="str">
-        <v>0.107s</v>
+        <v>0.122s</v>
       </c>
     </row>
     <row r="274">
@@ -5054,7 +5054,7 @@
         <v>HIGH</v>
       </c>
       <c r="E274" t="str">
-        <v>0.107s</v>
+        <v>0.129s</v>
       </c>
     </row>
     <row r="275">
@@ -5071,7 +5071,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E275" t="str">
-        <v>0.110s</v>
+        <v>0.067s</v>
       </c>
     </row>
     <row r="276">
@@ -5088,7 +5088,7 @@
         <v>LOW</v>
       </c>
       <c r="E276" t="str">
-        <v>0.075s</v>
+        <v>0.132s</v>
       </c>
     </row>
     <row r="277">
@@ -5105,7 +5105,7 @@
         <v>HIGH</v>
       </c>
       <c r="E277" t="str">
-        <v>0.149s</v>
+        <v>0.101s</v>
       </c>
     </row>
     <row r="278">
@@ -5122,7 +5122,7 @@
         <v>LOW</v>
       </c>
       <c r="E278" t="str">
-        <v>0.065s</v>
+        <v>0.049s</v>
       </c>
     </row>
     <row r="279">
@@ -5139,7 +5139,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E279" t="str">
-        <v>0.076s</v>
+        <v>0.091s</v>
       </c>
     </row>
     <row r="280">
@@ -5156,7 +5156,7 @@
         <v>LOW</v>
       </c>
       <c r="E280" t="str">
-        <v>0.063s</v>
+        <v>0.156s</v>
       </c>
     </row>
     <row r="281">
@@ -5173,7 +5173,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E281" t="str">
-        <v>0.099s</v>
+        <v>0.108s</v>
       </c>
     </row>
     <row r="282">
@@ -5190,7 +5190,7 @@
         <v>HIGH</v>
       </c>
       <c r="E282" t="str">
-        <v>0.049s</v>
+        <v>0.107s</v>
       </c>
     </row>
     <row r="283">
@@ -5207,7 +5207,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E283" t="str">
-        <v>0.073s</v>
+        <v>0.095s</v>
       </c>
     </row>
     <row r="284">
@@ -5224,7 +5224,7 @@
         <v>LOW</v>
       </c>
       <c r="E284" t="str">
-        <v>0.095s</v>
+        <v>0.046s</v>
       </c>
     </row>
     <row r="285">
@@ -5241,7 +5241,7 @@
         <v>HIGH</v>
       </c>
       <c r="E285" t="str">
-        <v>0.133s</v>
+        <v>0.094s</v>
       </c>
     </row>
     <row r="286">
@@ -5258,7 +5258,7 @@
         <v>LOW</v>
       </c>
       <c r="E286" t="str">
-        <v>0.087s</v>
+        <v>0.150s</v>
       </c>
     </row>
     <row r="287">
@@ -5275,7 +5275,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E287" t="str">
-        <v>0.110s</v>
+        <v>0.154s</v>
       </c>
     </row>
     <row r="288">
@@ -5292,7 +5292,7 @@
         <v>HIGH</v>
       </c>
       <c r="E288" t="str">
-        <v>0.111s</v>
+        <v>0.084s</v>
       </c>
     </row>
     <row r="289">
@@ -5309,7 +5309,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E289" t="str">
-        <v>0.110s</v>
+        <v>0.070s</v>
       </c>
     </row>
     <row r="290">
@@ -5326,7 +5326,7 @@
         <v>LOW</v>
       </c>
       <c r="E290" t="str">
-        <v>0.073s</v>
+        <v>0.070s</v>
       </c>
     </row>
     <row r="291">
@@ -5343,7 +5343,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E291" t="str">
-        <v>0.044s</v>
+        <v>0.051s</v>
       </c>
     </row>
     <row r="292">
@@ -5360,7 +5360,7 @@
         <v>LOW</v>
       </c>
       <c r="E292" t="str">
-        <v>0.060s</v>
+        <v>0.132s</v>
       </c>
     </row>
     <row r="293">
@@ -5377,7 +5377,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E293" t="str">
-        <v>0.052s</v>
+        <v>0.128s</v>
       </c>
     </row>
     <row r="294">
@@ -5394,7 +5394,7 @@
         <v>HIGH</v>
       </c>
       <c r="E294" t="str">
-        <v>0.111s</v>
+        <v>0.128s</v>
       </c>
     </row>
     <row r="295">
@@ -5411,7 +5411,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E295" t="str">
-        <v>0.104s</v>
+        <v>0.066s</v>
       </c>
     </row>
     <row r="296">
@@ -5428,7 +5428,7 @@
         <v>LOW</v>
       </c>
       <c r="E296" t="str">
-        <v>0.055s</v>
+        <v>0.095s</v>
       </c>
     </row>
     <row r="297">
@@ -5445,7 +5445,7 @@
         <v>HIGH</v>
       </c>
       <c r="E297" t="str">
-        <v>0.117s</v>
+        <v>0.135s</v>
       </c>
     </row>
     <row r="298">
@@ -5462,7 +5462,7 @@
         <v>LOW</v>
       </c>
       <c r="E298" t="str">
-        <v>0.110s</v>
+        <v>0.140s</v>
       </c>
     </row>
     <row r="299">
@@ -5479,7 +5479,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E299" t="str">
-        <v>0.106s</v>
+        <v>0.067s</v>
       </c>
     </row>
     <row r="300">
@@ -5496,7 +5496,7 @@
         <v>HIGH</v>
       </c>
       <c r="E300" t="str">
-        <v>0.058s</v>
+        <v>0.052s</v>
       </c>
     </row>
     <row r="301">
@@ -5513,7 +5513,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E301" t="str">
-        <v>0.049s</v>
+        <v>0.043s</v>
       </c>
     </row>
     <row r="302">
@@ -5530,7 +5530,7 @@
         <v>LOW</v>
       </c>
       <c r="E302" t="str">
-        <v>0.091s</v>
+        <v>0.121s</v>
       </c>
     </row>
     <row r="303">
@@ -5547,7 +5547,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E303" t="str">
-        <v>0.084s</v>
+        <v>0.090s</v>
       </c>
     </row>
     <row r="304">
@@ -5564,7 +5564,7 @@
         <v>LOW</v>
       </c>
       <c r="E304" t="str">
-        <v>0.077s</v>
+        <v>0.116s</v>
       </c>
     </row>
     <row r="305">
@@ -5581,7 +5581,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E305" t="str">
-        <v>0.137s</v>
+        <v>0.084s</v>
       </c>
     </row>
     <row r="306">
@@ -5598,7 +5598,7 @@
         <v>HIGH</v>
       </c>
       <c r="E306" t="str">
-        <v>0.105s</v>
+        <v>0.107s</v>
       </c>
     </row>
     <row r="307">
@@ -5615,7 +5615,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E307" t="str">
-        <v>0.040s</v>
+        <v>0.047s</v>
       </c>
     </row>
     <row r="308">
@@ -5632,7 +5632,7 @@
         <v>LOW</v>
       </c>
       <c r="E308" t="str">
-        <v>0.146s</v>
+        <v>0.110s</v>
       </c>
     </row>
     <row r="309">
@@ -5649,7 +5649,7 @@
         <v>HIGH</v>
       </c>
       <c r="E309" t="str">
-        <v>0.087s</v>
+        <v>0.158s</v>
       </c>
     </row>
     <row r="310">
@@ -5666,7 +5666,7 @@
         <v>LOW</v>
       </c>
       <c r="E310" t="str">
-        <v>0.068s</v>
+        <v>0.138s</v>
       </c>
     </row>
     <row r="311">
@@ -5683,7 +5683,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E311" t="str">
-        <v>0.049s</v>
+        <v>0.067s</v>
       </c>
     </row>
     <row r="312">
@@ -5700,7 +5700,7 @@
         <v>HIGH</v>
       </c>
       <c r="E312" t="str">
-        <v>0.158s</v>
+        <v>0.114s</v>
       </c>
     </row>
     <row r="313">
@@ -5717,7 +5717,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E313" t="str">
-        <v>0.126s</v>
+        <v>0.100s</v>
       </c>
     </row>
     <row r="314">
@@ -5734,7 +5734,7 @@
         <v>LOW</v>
       </c>
       <c r="E314" t="str">
-        <v>0.151s</v>
+        <v>0.085s</v>
       </c>
     </row>
     <row r="315">
@@ -5751,7 +5751,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E315" t="str">
-        <v>0.100s</v>
+        <v>0.074s</v>
       </c>
     </row>
     <row r="316">
@@ -5768,7 +5768,7 @@
         <v>LOW</v>
       </c>
       <c r="E316" t="str">
-        <v>0.096s</v>
+        <v>0.112s</v>
       </c>
     </row>
     <row r="317">
@@ -5785,7 +5785,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E317" t="str">
-        <v>0.048s</v>
+        <v>0.146s</v>
       </c>
     </row>
     <row r="318">
@@ -5802,7 +5802,7 @@
         <v>HIGH</v>
       </c>
       <c r="E318" t="str">
-        <v>0.076s</v>
+        <v>0.111s</v>
       </c>
     </row>
     <row r="319">
@@ -5819,7 +5819,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E319" t="str">
-        <v>0.158s</v>
+        <v>0.101s</v>
       </c>
     </row>
     <row r="320">
@@ -5836,7 +5836,7 @@
         <v>LOW</v>
       </c>
       <c r="E320" t="str">
-        <v>0.042s</v>
+        <v>0.095s</v>
       </c>
     </row>
     <row r="321">
@@ -5853,7 +5853,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E321" t="str">
-        <v>0.121s</v>
+        <v>0.071s</v>
       </c>
     </row>
     <row r="322">
@@ -5870,7 +5870,7 @@
         <v>HIGH</v>
       </c>
       <c r="E322" t="str">
-        <v>0.046s</v>
+        <v>0.055s</v>
       </c>
     </row>
     <row r="323">
@@ -5887,7 +5887,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E323" t="str">
-        <v>0.073s</v>
+        <v>0.128s</v>
       </c>
     </row>
     <row r="324">
@@ -5904,7 +5904,7 @@
         <v>LOW</v>
       </c>
       <c r="E324" t="str">
-        <v>0.110s</v>
+        <v>0.071s</v>
       </c>
     </row>
     <row r="325">
@@ -5921,7 +5921,7 @@
         <v>HIGH</v>
       </c>
       <c r="E325" t="str">
-        <v>0.124s</v>
+        <v>0.095s</v>
       </c>
     </row>
     <row r="326">
@@ -5938,7 +5938,7 @@
         <v>LOW</v>
       </c>
       <c r="E326" t="str">
-        <v>0.087s</v>
+        <v>0.047s</v>
       </c>
     </row>
     <row r="327">
@@ -5955,7 +5955,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E327" t="str">
-        <v>0.082s</v>
+        <v>0.090s</v>
       </c>
     </row>
     <row r="328">
@@ -5972,7 +5972,7 @@
         <v>HIGH</v>
       </c>
       <c r="E328" t="str">
-        <v>0.053s</v>
+        <v>0.113s</v>
       </c>
     </row>
     <row r="329">
@@ -5989,7 +5989,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E329" t="str">
-        <v>0.097s</v>
+        <v>0.081s</v>
       </c>
     </row>
     <row r="330">
@@ -6006,7 +6006,7 @@
         <v>LOW</v>
       </c>
       <c r="E330" t="str">
-        <v>0.090s</v>
+        <v>0.105s</v>
       </c>
     </row>
     <row r="331">
@@ -6023,7 +6023,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E331" t="str">
-        <v>0.154s</v>
+        <v>0.053s</v>
       </c>
     </row>
     <row r="332">
@@ -6040,7 +6040,7 @@
         <v>LOW</v>
       </c>
       <c r="E332" t="str">
-        <v>0.100s</v>
+        <v>0.046s</v>
       </c>
     </row>
     <row r="333">
@@ -6057,7 +6057,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E333" t="str">
-        <v>0.117s</v>
+        <v>0.074s</v>
       </c>
     </row>
     <row r="334">
@@ -6074,7 +6074,7 @@
         <v>HIGH</v>
       </c>
       <c r="E334" t="str">
-        <v>0.076s</v>
+        <v>0.125s</v>
       </c>
     </row>
     <row r="335">
@@ -6091,7 +6091,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E335" t="str">
-        <v>0.132s</v>
+        <v>0.074s</v>
       </c>
     </row>
     <row r="336">
@@ -6108,7 +6108,7 @@
         <v>LOW</v>
       </c>
       <c r="E336" t="str">
-        <v>0.151s</v>
+        <v>0.131s</v>
       </c>
     </row>
     <row r="337">
@@ -6125,7 +6125,7 @@
         <v>HIGH</v>
       </c>
       <c r="E337" t="str">
-        <v>0.140s</v>
+        <v>0.074s</v>
       </c>
     </row>
     <row r="338">
@@ -6142,7 +6142,7 @@
         <v>LOW</v>
       </c>
       <c r="E338" t="str">
-        <v>0.155s</v>
+        <v>0.141s</v>
       </c>
     </row>
     <row r="339">
@@ -6159,7 +6159,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E339" t="str">
-        <v>0.042s</v>
+        <v>0.105s</v>
       </c>
     </row>
     <row r="340">
@@ -6176,7 +6176,7 @@
         <v>LOW</v>
       </c>
       <c r="E340" t="str">
-        <v>0.117s</v>
+        <v>0.078s</v>
       </c>
     </row>
     <row r="341">
@@ -6193,7 +6193,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E341" t="str">
-        <v>0.122s</v>
+        <v>0.048s</v>
       </c>
     </row>
     <row r="342">
@@ -6210,7 +6210,7 @@
         <v>HIGH</v>
       </c>
       <c r="E342" t="str">
-        <v>0.055s</v>
+        <v>0.068s</v>
       </c>
     </row>
     <row r="343">
@@ -6227,7 +6227,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E343" t="str">
-        <v>0.065s</v>
+        <v>0.076s</v>
       </c>
     </row>
     <row r="344">
@@ -6244,7 +6244,7 @@
         <v>LOW</v>
       </c>
       <c r="E344" t="str">
-        <v>0.076s</v>
+        <v>0.073s</v>
       </c>
     </row>
     <row r="345">
@@ -6261,7 +6261,7 @@
         <v>HIGH</v>
       </c>
       <c r="E345" t="str">
-        <v>0.134s</v>
+        <v>0.119s</v>
       </c>
     </row>
     <row r="346">
@@ -6278,7 +6278,7 @@
         <v>LOW</v>
       </c>
       <c r="E346" t="str">
-        <v>0.070s</v>
+        <v>0.131s</v>
       </c>
     </row>
     <row r="347">
@@ -6295,7 +6295,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E347" t="str">
-        <v>0.071s</v>
+        <v>0.150s</v>
       </c>
     </row>
     <row r="348">
@@ -6312,7 +6312,7 @@
         <v>HIGH</v>
       </c>
       <c r="E348" t="str">
-        <v>0.044s</v>
+        <v>0.108s</v>
       </c>
     </row>
     <row r="349">
@@ -6329,7 +6329,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E349" t="str">
-        <v>0.129s</v>
+        <v>0.120s</v>
       </c>
     </row>
     <row r="350">
@@ -6346,7 +6346,7 @@
         <v>LOW</v>
       </c>
       <c r="E350" t="str">
-        <v>0.083s</v>
+        <v>0.053s</v>
       </c>
     </row>
     <row r="351">
@@ -6363,7 +6363,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E351" t="str">
-        <v>0.099s</v>
+        <v>0.119s</v>
       </c>
     </row>
     <row r="352">
@@ -6380,7 +6380,7 @@
         <v>LOW</v>
       </c>
       <c r="E352" t="str">
-        <v>0.058s</v>
+        <v>0.150s</v>
       </c>
     </row>
     <row r="353">
@@ -6397,7 +6397,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E353" t="str">
-        <v>0.077s</v>
+        <v>0.072s</v>
       </c>
     </row>
     <row r="354">
@@ -6414,7 +6414,7 @@
         <v>HIGH</v>
       </c>
       <c r="E354" t="str">
-        <v>0.056s</v>
+        <v>0.085s</v>
       </c>
     </row>
     <row r="355">
@@ -6431,7 +6431,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E355" t="str">
-        <v>0.109s</v>
+        <v>0.145s</v>
       </c>
     </row>
     <row r="356">
@@ -6448,7 +6448,7 @@
         <v>LOW</v>
       </c>
       <c r="E356" t="str">
-        <v>0.148s</v>
+        <v>0.124s</v>
       </c>
     </row>
     <row r="357">
@@ -6465,7 +6465,7 @@
         <v>HIGH</v>
       </c>
       <c r="E357" t="str">
-        <v>0.040s</v>
+        <v>0.082s</v>
       </c>
     </row>
     <row r="358">
@@ -6482,7 +6482,7 @@
         <v>LOW</v>
       </c>
       <c r="E358" t="str">
-        <v>0.119s</v>
+        <v>0.090s</v>
       </c>
     </row>
     <row r="359">
@@ -6499,7 +6499,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E359" t="str">
-        <v>0.040s</v>
+        <v>0.103s</v>
       </c>
     </row>
     <row r="360">
@@ -6516,7 +6516,7 @@
         <v>LOW</v>
       </c>
       <c r="E360" t="str">
-        <v>0.134s</v>
+        <v>0.047s</v>
       </c>
     </row>
     <row r="361">
@@ -6533,7 +6533,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E361" t="str">
-        <v>0.106s</v>
+        <v>0.098s</v>
       </c>
     </row>
     <row r="362">
@@ -6550,7 +6550,7 @@
         <v>HIGH</v>
       </c>
       <c r="E362" t="str">
-        <v>0.091s</v>
+        <v>0.153s</v>
       </c>
     </row>
     <row r="363">
@@ -6567,7 +6567,7 @@
         <v>LOW</v>
       </c>
       <c r="E363" t="str">
-        <v>0.131s</v>
+        <v>0.065s</v>
       </c>
     </row>
     <row r="364">
@@ -6584,7 +6584,7 @@
         <v>HIGH</v>
       </c>
       <c r="E364" t="str">
-        <v>0.063s</v>
+        <v>0.098s</v>
       </c>
     </row>
     <row r="365">
@@ -6601,7 +6601,7 @@
         <v>LOW</v>
       </c>
       <c r="E365" t="str">
-        <v>0.146s</v>
+        <v>0.134s</v>
       </c>
     </row>
     <row r="366">
@@ -6618,7 +6618,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E366" t="str">
-        <v>0.154s</v>
+        <v>0.065s</v>
       </c>
     </row>
     <row r="367">
@@ -6635,7 +6635,7 @@
         <v>HIGH</v>
       </c>
       <c r="E367" t="str">
-        <v>0.083s</v>
+        <v>0.050s</v>
       </c>
     </row>
     <row r="368">
@@ -6652,7 +6652,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E368" t="str">
-        <v>0.135s</v>
+        <v>0.047s</v>
       </c>
     </row>
     <row r="369">
@@ -6669,7 +6669,7 @@
         <v>LOW</v>
       </c>
       <c r="E369" t="str">
-        <v>0.050s</v>
+        <v>0.097s</v>
       </c>
     </row>
     <row r="370">
@@ -6686,7 +6686,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E370" t="str">
-        <v>0.135s</v>
+        <v>0.091s</v>
       </c>
     </row>
     <row r="371">
@@ -6703,7 +6703,7 @@
         <v>LOW</v>
       </c>
       <c r="E371" t="str">
-        <v>0.128s</v>
+        <v>0.130s</v>
       </c>
     </row>
     <row r="372">
@@ -6720,7 +6720,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E372" t="str">
-        <v>0.141s</v>
+        <v>0.068s</v>
       </c>
     </row>
     <row r="373">
@@ -6737,7 +6737,7 @@
         <v>HIGH</v>
       </c>
       <c r="E373" t="str">
-        <v>0.110s</v>
+        <v>0.147s</v>
       </c>
     </row>
     <row r="374">
@@ -6754,7 +6754,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E374" t="str">
-        <v>0.047s</v>
+        <v>0.117s</v>
       </c>
     </row>
     <row r="375">
@@ -6771,7 +6771,7 @@
         <v>LOW</v>
       </c>
       <c r="E375" t="str">
-        <v>0.123s</v>
+        <v>0.104s</v>
       </c>
     </row>
     <row r="376">
@@ -6788,7 +6788,7 @@
         <v>HIGH</v>
       </c>
       <c r="E376" t="str">
-        <v>0.132s</v>
+        <v>0.150s</v>
       </c>
     </row>
     <row r="377">
@@ -6805,7 +6805,7 @@
         <v>LOW</v>
       </c>
       <c r="E377" t="str">
-        <v>0.064s</v>
+        <v>0.082s</v>
       </c>
     </row>
     <row r="378">
@@ -6822,7 +6822,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E378" t="str">
-        <v>0.072s</v>
+        <v>0.120s</v>
       </c>
     </row>
     <row r="379">
@@ -6839,7 +6839,7 @@
         <v>LOW</v>
       </c>
       <c r="E379" t="str">
-        <v>0.157s</v>
+        <v>0.048s</v>
       </c>
     </row>
     <row r="380">
@@ -6856,7 +6856,7 @@
         <v>HIGH</v>
       </c>
       <c r="E380" t="str">
-        <v>0.160s</v>
+        <v>0.123s</v>
       </c>
     </row>
     <row r="381">
@@ -6873,7 +6873,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E381" t="str">
-        <v>0.128s</v>
+        <v>0.138s</v>
       </c>
     </row>
     <row r="382">
@@ -6890,7 +6890,7 @@
         <v>LOW</v>
       </c>
       <c r="E382" t="str">
-        <v>0.066s</v>
+        <v>0.111s</v>
       </c>
     </row>
     <row r="383">
@@ -6907,7 +6907,7 @@
         <v>HIGH</v>
       </c>
       <c r="E383" t="str">
-        <v>0.056s</v>
+        <v>0.148s</v>
       </c>
     </row>
     <row r="384">
@@ -6924,7 +6924,7 @@
         <v>LOW</v>
       </c>
       <c r="E384" t="str">
-        <v>0.116s</v>
+        <v>0.047s</v>
       </c>
     </row>
     <row r="385">
@@ -6941,7 +6941,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E385" t="str">
-        <v>0.155s</v>
+        <v>0.117s</v>
       </c>
     </row>
     <row r="386">
@@ -6958,7 +6958,7 @@
         <v>HIGH</v>
       </c>
       <c r="E386" t="str">
-        <v>0.073s</v>
+        <v>0.127s</v>
       </c>
     </row>
     <row r="387">
@@ -6975,7 +6975,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E387" t="str">
-        <v>0.125s</v>
+        <v>0.084s</v>
       </c>
     </row>
     <row r="388">
@@ -6992,7 +6992,7 @@
         <v>LOW</v>
       </c>
       <c r="E388" t="str">
-        <v>0.117s</v>
+        <v>0.131s</v>
       </c>
     </row>
     <row r="389">
@@ -7009,7 +7009,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E389" t="str">
-        <v>0.062s</v>
+        <v>0.150s</v>
       </c>
     </row>
     <row r="390">
@@ -7026,7 +7026,7 @@
         <v>LOW</v>
       </c>
       <c r="E390" t="str">
-        <v>0.079s</v>
+        <v>0.070s</v>
       </c>
     </row>
     <row r="391">
@@ -7043,7 +7043,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E391" t="str">
-        <v>0.160s</v>
+        <v>0.104s</v>
       </c>
     </row>
     <row r="392">
@@ -7060,7 +7060,7 @@
         <v>HIGH</v>
       </c>
       <c r="E392" t="str">
-        <v>0.075s</v>
+        <v>0.120s</v>
       </c>
     </row>
     <row r="393">
@@ -7077,7 +7077,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E393" t="str">
-        <v>0.143s</v>
+        <v>0.079s</v>
       </c>
     </row>
     <row r="394">
@@ -7094,7 +7094,7 @@
         <v>LOW</v>
       </c>
       <c r="E394" t="str">
-        <v>0.105s</v>
+        <v>0.133s</v>
       </c>
     </row>
     <row r="395">
@@ -7111,7 +7111,7 @@
         <v>HIGH</v>
       </c>
       <c r="E395" t="str">
-        <v>0.143s</v>
+        <v>0.113s</v>
       </c>
     </row>
     <row r="396">
@@ -7128,7 +7128,7 @@
         <v>LOW</v>
       </c>
       <c r="E396" t="str">
-        <v>0.050s</v>
+        <v>0.067s</v>
       </c>
     </row>
     <row r="397">
@@ -7145,7 +7145,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E397" t="str">
-        <v>0.138s</v>
+        <v>0.119s</v>
       </c>
     </row>
     <row r="398">
@@ -7162,7 +7162,7 @@
         <v>LOW</v>
       </c>
       <c r="E398" t="str">
-        <v>0.120s</v>
+        <v>0.097s</v>
       </c>
     </row>
     <row r="399">
@@ -7179,7 +7179,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E399" t="str">
-        <v>0.109s</v>
+        <v>0.054s</v>
       </c>
     </row>
     <row r="400">
@@ -7196,7 +7196,7 @@
         <v>HIGH</v>
       </c>
       <c r="E400" t="str">
-        <v>0.078s</v>
+        <v>0.061s</v>
       </c>
     </row>
     <row r="401">
@@ -7213,7 +7213,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E401" t="str">
-        <v>0.125s</v>
+        <v>0.109s</v>
       </c>
     </row>
     <row r="402">
@@ -7230,7 +7230,7 @@
         <v>LOW</v>
       </c>
       <c r="E402" t="str">
-        <v>0.096s</v>
+        <v>0.057s</v>
       </c>
     </row>
     <row r="403">
@@ -7247,7 +7247,7 @@
         <v>HIGH</v>
       </c>
       <c r="E403" t="str">
-        <v>0.060s</v>
+        <v>0.064s</v>
       </c>
     </row>
     <row r="404">
@@ -7264,7 +7264,7 @@
         <v>LOW</v>
       </c>
       <c r="E404" t="str">
-        <v>0.092s</v>
+        <v>0.112s</v>
       </c>
     </row>
     <row r="405">
@@ -7281,7 +7281,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E405" t="str">
-        <v>0.100s</v>
+        <v>0.118s</v>
       </c>
     </row>
     <row r="406">
@@ -7298,7 +7298,7 @@
         <v>HIGH</v>
       </c>
       <c r="E406" t="str">
-        <v>0.130s</v>
+        <v>0.104s</v>
       </c>
     </row>
     <row r="407">
@@ -7315,7 +7315,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E407" t="str">
-        <v>0.130s</v>
+        <v>0.110s</v>
       </c>
     </row>
     <row r="408">
@@ -7332,7 +7332,7 @@
         <v>LOW</v>
       </c>
       <c r="E408" t="str">
-        <v>0.107s</v>
+        <v>0.089s</v>
       </c>
     </row>
     <row r="409">
@@ -7349,7 +7349,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E409" t="str">
-        <v>0.045s</v>
+        <v>0.080s</v>
       </c>
     </row>
     <row r="410">
@@ -7366,7 +7366,7 @@
         <v>HIGH</v>
       </c>
       <c r="E410" t="str">
-        <v>0.047s</v>
+        <v>0.109s</v>
       </c>
     </row>
     <row r="411">
@@ -7383,7 +7383,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E411" t="str">
-        <v>0.130s</v>
+        <v>0.054s</v>
       </c>
     </row>
     <row r="412">
@@ -7400,7 +7400,7 @@
         <v>LOW</v>
       </c>
       <c r="E412" t="str">
-        <v>0.138s</v>
+        <v>0.142s</v>
       </c>
     </row>
     <row r="413">
@@ -7417,7 +7417,7 @@
         <v>HIGH</v>
       </c>
       <c r="E413" t="str">
-        <v>0.142s</v>
+        <v>0.056s</v>
       </c>
     </row>
     <row r="414">
@@ -7434,7 +7434,7 @@
         <v>LOW</v>
       </c>
       <c r="E414" t="str">
-        <v>0.091s</v>
+        <v>0.135s</v>
       </c>
     </row>
     <row r="415">
@@ -7451,7 +7451,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E415" t="str">
-        <v>0.131s</v>
+        <v>0.058s</v>
       </c>
     </row>
     <row r="416">
@@ -7468,7 +7468,7 @@
         <v>HIGH</v>
       </c>
       <c r="E416" t="str">
-        <v>0.143s</v>
+        <v>0.137s</v>
       </c>
     </row>
     <row r="417">
@@ -7485,7 +7485,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E417" t="str">
-        <v>0.043s</v>
+        <v>0.088s</v>
       </c>
     </row>
     <row r="418">
@@ -7502,7 +7502,7 @@
         <v>LOW</v>
       </c>
       <c r="E418" t="str">
-        <v>0.152s</v>
+        <v>0.119s</v>
       </c>
     </row>
     <row r="419">
@@ -7519,7 +7519,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E419" t="str">
-        <v>0.083s</v>
+        <v>0.127s</v>
       </c>
     </row>
     <row r="420">
@@ -7536,7 +7536,7 @@
         <v>LOW</v>
       </c>
       <c r="E420" t="str">
-        <v>0.084s</v>
+        <v>0.096s</v>
       </c>
     </row>
     <row r="421">
@@ -7553,7 +7553,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E421" t="str">
-        <v>0.071s</v>
+        <v>0.132s</v>
       </c>
     </row>
     <row r="422">
@@ -7570,7 +7570,7 @@
         <v>HIGH</v>
       </c>
       <c r="E422" t="str">
-        <v>0.125s</v>
+        <v>0.128s</v>
       </c>
     </row>
     <row r="423">
@@ -7587,7 +7587,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E423" t="str">
-        <v>0.105s</v>
+        <v>0.088s</v>
       </c>
     </row>
     <row r="424">
@@ -7604,7 +7604,7 @@
         <v>LOW</v>
       </c>
       <c r="E424" t="str">
-        <v>0.124s</v>
+        <v>0.079s</v>
       </c>
     </row>
     <row r="425">
@@ -7621,7 +7621,7 @@
         <v>HIGH</v>
       </c>
       <c r="E425" t="str">
-        <v>0.081s</v>
+        <v>0.078s</v>
       </c>
     </row>
     <row r="426">
@@ -7638,7 +7638,7 @@
         <v>LOW</v>
       </c>
       <c r="E426" t="str">
-        <v>0.136s</v>
+        <v>0.091s</v>
       </c>
     </row>
     <row r="427">
@@ -7655,7 +7655,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E427" t="str">
-        <v>0.059s</v>
+        <v>0.103s</v>
       </c>
     </row>
     <row r="428">
@@ -7672,7 +7672,7 @@
         <v>LOW</v>
       </c>
       <c r="E428" t="str">
-        <v>0.085s</v>
+        <v>0.127s</v>
       </c>
     </row>
     <row r="429">
@@ -7689,7 +7689,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E429" t="str">
-        <v>0.113s</v>
+        <v>0.044s</v>
       </c>
     </row>
     <row r="430">
@@ -7706,7 +7706,7 @@
         <v>HIGH</v>
       </c>
       <c r="E430" t="str">
-        <v>0.043s</v>
+        <v>0.126s</v>
       </c>
     </row>
     <row r="431">
@@ -7723,7 +7723,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E431" t="str">
-        <v>0.087s</v>
+        <v>0.053s</v>
       </c>
     </row>
     <row r="432">
@@ -7740,7 +7740,7 @@
         <v>LOW</v>
       </c>
       <c r="E432" t="str">
-        <v>0.059s</v>
+        <v>0.139s</v>
       </c>
     </row>
     <row r="433">
@@ -7757,7 +7757,7 @@
         <v>HIGH</v>
       </c>
       <c r="E433" t="str">
-        <v>0.062s</v>
+        <v>0.110s</v>
       </c>
     </row>
     <row r="434">
@@ -7774,7 +7774,7 @@
         <v>LOW</v>
       </c>
       <c r="E434" t="str">
-        <v>0.070s</v>
+        <v>0.054s</v>
       </c>
     </row>
     <row r="435">
@@ -7791,7 +7791,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E435" t="str">
-        <v>0.097s</v>
+        <v>0.068s</v>
       </c>
     </row>
     <row r="436">
@@ -7808,7 +7808,7 @@
         <v>HIGH</v>
       </c>
       <c r="E436" t="str">
-        <v>0.070s</v>
+        <v>0.082s</v>
       </c>
     </row>
     <row r="437">
@@ -7825,7 +7825,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E437" t="str">
-        <v>0.095s</v>
+        <v>0.060s</v>
       </c>
     </row>
     <row r="438">
@@ -7842,7 +7842,7 @@
         <v>LOW</v>
       </c>
       <c r="E438" t="str">
-        <v>0.145s</v>
+        <v>0.127s</v>
       </c>
     </row>
     <row r="439">
@@ -7859,7 +7859,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E439" t="str">
-        <v>0.130s</v>
+        <v>0.088s</v>
       </c>
     </row>
     <row r="440">
@@ -7876,7 +7876,7 @@
         <v>HIGH</v>
       </c>
       <c r="E440" t="str">
-        <v>0.154s</v>
+        <v>0.121s</v>
       </c>
     </row>
     <row r="441">
@@ -7893,7 +7893,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E441" t="str">
-        <v>0.074s</v>
+        <v>0.132s</v>
       </c>
     </row>
     <row r="442">
@@ -7910,7 +7910,7 @@
         <v>LOW</v>
       </c>
       <c r="E442" t="str">
-        <v>0.065s</v>
+        <v>0.128s</v>
       </c>
     </row>
     <row r="443">
@@ -7927,7 +7927,7 @@
         <v>HIGH</v>
       </c>
       <c r="E443" t="str">
-        <v>0.057s</v>
+        <v>0.116s</v>
       </c>
     </row>
     <row r="444">
@@ -7944,7 +7944,7 @@
         <v>LOW</v>
       </c>
       <c r="E444" t="str">
-        <v>0.093s</v>
+        <v>0.157s</v>
       </c>
     </row>
     <row r="445">
@@ -7961,7 +7961,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E445" t="str">
-        <v>0.154s</v>
+        <v>0.062s</v>
       </c>
     </row>
     <row r="446">
@@ -7995,7 +7995,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E447" t="str">
-        <v>0.157s</v>
+        <v>0.123s</v>
       </c>
     </row>
     <row r="448">
@@ -8012,7 +8012,7 @@
         <v>LOW</v>
       </c>
       <c r="E448" t="str">
-        <v>0.067s</v>
+        <v>0.100s</v>
       </c>
     </row>
     <row r="449">
@@ -8029,7 +8029,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E449" t="str">
-        <v>0.062s</v>
+        <v>0.128s</v>
       </c>
     </row>
     <row r="450">
@@ -8046,7 +8046,7 @@
         <v>LOW</v>
       </c>
       <c r="E450" t="str">
-        <v>0.159s</v>
+        <v>0.150s</v>
       </c>
     </row>
     <row r="451">
@@ -8063,7 +8063,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E451" t="str">
-        <v>0.151s</v>
+        <v>0.127s</v>
       </c>
     </row>
     <row r="452">
@@ -8080,7 +8080,7 @@
         <v>HIGH</v>
       </c>
       <c r="E452" t="str">
-        <v>0.138s</v>
+        <v>0.082s</v>
       </c>
     </row>
     <row r="453">
@@ -8097,7 +8097,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E453" t="str">
-        <v>0.087s</v>
+        <v>0.070s</v>
       </c>
     </row>
     <row r="454">
@@ -8114,7 +8114,7 @@
         <v>LOW</v>
       </c>
       <c r="E454" t="str">
-        <v>0.105s</v>
+        <v>0.148s</v>
       </c>
     </row>
     <row r="455">
@@ -8131,7 +8131,7 @@
         <v>HIGH</v>
       </c>
       <c r="E455" t="str">
-        <v>0.078s</v>
+        <v>0.096s</v>
       </c>
     </row>
     <row r="456">
@@ -8148,7 +8148,7 @@
         <v>LOW</v>
       </c>
       <c r="E456" t="str">
-        <v>0.096s</v>
+        <v>0.156s</v>
       </c>
     </row>
     <row r="457">
@@ -8165,7 +8165,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E457" t="str">
-        <v>0.107s</v>
+        <v>0.140s</v>
       </c>
     </row>
     <row r="458">
@@ -8182,7 +8182,7 @@
         <v>LOW</v>
       </c>
       <c r="E458" t="str">
-        <v>0.098s</v>
+        <v>0.153s</v>
       </c>
     </row>
     <row r="459">
@@ -8199,7 +8199,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E459" t="str">
-        <v>0.096s</v>
+        <v>0.151s</v>
       </c>
     </row>
     <row r="460">
@@ -8216,7 +8216,7 @@
         <v>HIGH</v>
       </c>
       <c r="E460" t="str">
-        <v>0.158s</v>
+        <v>0.124s</v>
       </c>
     </row>
     <row r="461">
@@ -8233,7 +8233,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E461" t="str">
-        <v>0.108s</v>
+        <v>0.137s</v>
       </c>
     </row>
     <row r="462">
@@ -8250,7 +8250,7 @@
         <v>LOW</v>
       </c>
       <c r="E462" t="str">
-        <v>0.091s</v>
+        <v>0.154s</v>
       </c>
     </row>
     <row r="463">
@@ -8267,7 +8267,7 @@
         <v>HIGH</v>
       </c>
       <c r="E463" t="str">
-        <v>0.081s</v>
+        <v>0.077s</v>
       </c>
     </row>
     <row r="464">
@@ -8284,7 +8284,7 @@
         <v>LOW</v>
       </c>
       <c r="E464" t="str">
-        <v>0.154s</v>
+        <v>0.115s</v>
       </c>
     </row>
     <row r="465">
@@ -8301,7 +8301,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E465" t="str">
-        <v>0.074s</v>
+        <v>0.103s</v>
       </c>
     </row>
     <row r="466">
@@ -8318,7 +8318,7 @@
         <v>HIGH</v>
       </c>
       <c r="E466" t="str">
-        <v>0.045s</v>
+        <v>0.087s</v>
       </c>
     </row>
     <row r="467">
@@ -8335,7 +8335,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E467" t="str">
-        <v>0.050s</v>
+        <v>0.141s</v>
       </c>
     </row>
     <row r="468">
@@ -8352,7 +8352,7 @@
         <v>LOW</v>
       </c>
       <c r="E468" t="str">
-        <v>0.061s</v>
+        <v>0.151s</v>
       </c>
     </row>
     <row r="469">
@@ -8369,7 +8369,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E469" t="str">
-        <v>0.067s</v>
+        <v>0.097s</v>
       </c>
     </row>
     <row r="470">
@@ -8386,7 +8386,7 @@
         <v>LOW</v>
       </c>
       <c r="E470" t="str">
-        <v>0.107s</v>
+        <v>0.064s</v>
       </c>
     </row>
     <row r="471">
@@ -8403,7 +8403,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E471" t="str">
-        <v>0.067s</v>
+        <v>0.148s</v>
       </c>
     </row>
     <row r="472">
@@ -8420,7 +8420,7 @@
         <v>HIGH</v>
       </c>
       <c r="E472" t="str">
-        <v>0.125s</v>
+        <v>0.072s</v>
       </c>
     </row>
     <row r="473">
@@ -8437,7 +8437,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E473" t="str">
-        <v>0.145s</v>
+        <v>0.107s</v>
       </c>
     </row>
     <row r="474">
@@ -8454,7 +8454,7 @@
         <v>LOW</v>
       </c>
       <c r="E474" t="str">
-        <v>0.147s</v>
+        <v>0.041s</v>
       </c>
     </row>
     <row r="475">
@@ -8471,7 +8471,7 @@
         <v>HIGH</v>
       </c>
       <c r="E475" t="str">
-        <v>0.062s</v>
+        <v>0.058s</v>
       </c>
     </row>
     <row r="476">
@@ -8488,7 +8488,7 @@
         <v>LOW</v>
       </c>
       <c r="E476" t="str">
-        <v>0.092s</v>
+        <v>0.064s</v>
       </c>
     </row>
     <row r="477">
@@ -8505,7 +8505,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E477" t="str">
-        <v>0.141s</v>
+        <v>0.081s</v>
       </c>
     </row>
     <row r="478">
@@ -8522,7 +8522,7 @@
         <v>HIGH</v>
       </c>
       <c r="E478" t="str">
-        <v>0.073s</v>
+        <v>0.147s</v>
       </c>
     </row>
     <row r="479">
@@ -8539,7 +8539,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E479" t="str">
-        <v>0.101s</v>
+        <v>0.140s</v>
       </c>
     </row>
     <row r="480">
@@ -8556,7 +8556,7 @@
         <v>LOW</v>
       </c>
       <c r="E480" t="str">
-        <v>0.081s</v>
+        <v>0.046s</v>
       </c>
     </row>
     <row r="481">
@@ -8573,7 +8573,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E481" t="str">
-        <v>0.063s</v>
+        <v>0.081s</v>
       </c>
     </row>
     <row r="482">
@@ -8590,7 +8590,7 @@
         <v>LOW</v>
       </c>
       <c r="E482" t="str">
-        <v>0.145s</v>
+        <v>0.103s</v>
       </c>
     </row>
     <row r="483">
@@ -8607,7 +8607,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E483" t="str">
-        <v>0.075s</v>
+        <v>0.073s</v>
       </c>
     </row>
     <row r="484">
@@ -8624,7 +8624,7 @@
         <v>HIGH</v>
       </c>
       <c r="E484" t="str">
-        <v>0.068s</v>
+        <v>0.094s</v>
       </c>
     </row>
     <row r="485">
@@ -8641,7 +8641,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E485" t="str">
-        <v>0.156s</v>
+        <v>0.047s</v>
       </c>
     </row>
     <row r="486">
@@ -8658,7 +8658,7 @@
         <v>LOW</v>
       </c>
       <c r="E486" t="str">
-        <v>0.156s</v>
+        <v>0.077s</v>
       </c>
     </row>
     <row r="487">
@@ -8675,7 +8675,7 @@
         <v>HIGH</v>
       </c>
       <c r="E487" t="str">
-        <v>0.090s</v>
+        <v>0.124s</v>
       </c>
     </row>
     <row r="488">
@@ -8692,7 +8692,7 @@
         <v>LOW</v>
       </c>
       <c r="E488" t="str">
-        <v>0.122s</v>
+        <v>0.044s</v>
       </c>
     </row>
     <row r="489">
@@ -8709,7 +8709,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E489" t="str">
-        <v>0.069s</v>
+        <v>0.155s</v>
       </c>
     </row>
     <row r="490">
@@ -8726,7 +8726,7 @@
         <v>HIGH</v>
       </c>
       <c r="E490" t="str">
-        <v>0.098s</v>
+        <v>0.076s</v>
       </c>
     </row>
     <row r="491">
@@ -8743,7 +8743,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E491" t="str">
-        <v>0.069s</v>
+        <v>0.091s</v>
       </c>
     </row>
     <row r="492">
@@ -8760,7 +8760,7 @@
         <v>LOW</v>
       </c>
       <c r="E492" t="str">
-        <v>0.050s</v>
+        <v>0.091s</v>
       </c>
     </row>
     <row r="493">
@@ -8777,7 +8777,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E493" t="str">
-        <v>0.056s</v>
+        <v>0.052s</v>
       </c>
     </row>
     <row r="494">
@@ -8794,7 +8794,7 @@
         <v>LOW</v>
       </c>
       <c r="E494" t="str">
-        <v>0.090s</v>
+        <v>0.133s</v>
       </c>
     </row>
     <row r="495">
@@ -8811,7 +8811,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E495" t="str">
-        <v>0.098s</v>
+        <v>0.074s</v>
       </c>
     </row>
     <row r="496">
@@ -8828,7 +8828,7 @@
         <v>HIGH</v>
       </c>
       <c r="E496" t="str">
-        <v>0.146s</v>
+        <v>0.117s</v>
       </c>
     </row>
     <row r="497">
@@ -8845,7 +8845,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E497" t="str">
-        <v>0.140s</v>
+        <v>0.083s</v>
       </c>
     </row>
     <row r="498">
@@ -8862,7 +8862,7 @@
         <v>LOW</v>
       </c>
       <c r="E498" t="str">
-        <v>0.081s</v>
+        <v>0.094s</v>
       </c>
     </row>
     <row r="499">
@@ -8879,7 +8879,7 @@
         <v>HIGH</v>
       </c>
       <c r="E499" t="str">
-        <v>0.102s</v>
+        <v>0.080s</v>
       </c>
     </row>
     <row r="500">
@@ -8896,7 +8896,7 @@
         <v>LOW</v>
       </c>
       <c r="E500" t="str">
-        <v>0.141s</v>
+        <v>0.125s</v>
       </c>
     </row>
     <row r="501">
@@ -8913,7 +8913,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E501" t="str">
-        <v>0.069s</v>
+        <v>0.095s</v>
       </c>
     </row>
     <row r="502">
@@ -8930,7 +8930,7 @@
         <v>HIGH</v>
       </c>
       <c r="E502" t="str">
-        <v>0.159s</v>
+        <v>0.141s</v>
       </c>
     </row>
     <row r="503">
@@ -8947,7 +8947,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E503" t="str">
-        <v>0.074s</v>
+        <v>0.141s</v>
       </c>
     </row>
     <row r="504">
@@ -8964,7 +8964,7 @@
         <v>LOW</v>
       </c>
       <c r="E504" t="str">
-        <v>0.125s</v>
+        <v>0.103s</v>
       </c>
     </row>
     <row r="505">
@@ -8981,7 +8981,7 @@
         <v>CRITICAL</v>
       </c>
       <c r="E505" t="str">
-        <v>0.041s</v>
+        <v>0.098s</v>
       </c>
     </row>
     <row r="506">
@@ -8998,7 +8998,7 @@
         <v>LOW</v>
       </c>
       <c r="E506" t="str">
-        <v>0.126s</v>
+        <v>0.053s</v>
       </c>
     </row>
     <row r="507">
@@ -9015,7 +9015,7 @@
         <v>MEDIUM</v>
       </c>
       <c r="E507" t="str">
-        <v>0.139s</v>
+        <v>0.138s</v>
       </c>
     </row>
   </sheetData>

</xml_diff>